<commit_message>
Remove 4 non-valve items from structure
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019oxoH766RXuqLqXQEjeJHj
</commit_message>
<xml_diff>
--- a/Estrutura_04.01.3.000598.xlsx
+++ b/Estrutura_04.01.3.000598.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I113"/>
+  <dimension ref="A1:I109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -494,7 +494,6 @@
       <c r="A2" t="n">
         <v>0</v>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
           <t>04.01.3.000598</t>
@@ -505,15 +504,12 @@
           <t>VÁLVULA BORBOLETA DUPLA ALAVANCA DN 700 .</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
         <v>1</v>
       </c>
       <c r="G2" t="n">
         <v>1</v>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -586,8 +582,6 @@
       <c r="G4" t="n">
         <v>1</v>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -619,8 +613,6 @@
       <c r="G5" t="n">
         <v>1</v>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -652,8 +644,6 @@
       <c r="G6" t="n">
         <v>1</v>
       </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -685,8 +675,6 @@
       <c r="G7" t="n">
         <v>2</v>
       </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -718,8 +706,6 @@
       <c r="G8" t="n">
         <v>2</v>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -751,8 +737,6 @@
       <c r="G9" t="n">
         <v>1</v>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -784,8 +768,6 @@
       <c r="G10" t="n">
         <v>1</v>
       </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -817,8 +799,6 @@
       <c r="G11" t="n">
         <v>1</v>
       </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -850,8 +830,6 @@
       <c r="G12" t="n">
         <v>2</v>
       </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -883,8 +861,6 @@
       <c r="G13" t="n">
         <v>2</v>
       </c>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -916,8 +892,6 @@
       <c r="G14" t="n">
         <v>2</v>
       </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -949,8 +923,6 @@
       <c r="G15" t="n">
         <v>2</v>
       </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -982,8 +954,6 @@
       <c r="G16" t="n">
         <v>2</v>
       </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1015,8 +985,6 @@
       <c r="G17" t="n">
         <v>4</v>
       </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1048,8 +1016,6 @@
       <c r="G18" t="n">
         <v>4</v>
       </c>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1086,7 +1052,6 @@
           <t>ASTM A36</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1123,7 +1088,6 @@
           <t>ASTM A516 GR70</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1160,7 +1124,6 @@
           <t>AISI 304</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1197,7 +1160,6 @@
           <t>AISI 304</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1234,7 +1196,6 @@
           <t>ASTM A516 GR70</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1266,8 +1227,6 @@
       <c r="G24" t="n">
         <v>2</v>
       </c>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1299,8 +1258,6 @@
       <c r="G25" t="n">
         <v>2</v>
       </c>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1332,8 +1289,6 @@
       <c r="G26" t="n">
         <v>2</v>
       </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1365,8 +1320,6 @@
       <c r="G27" t="n">
         <v>4</v>
       </c>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1403,7 +1356,6 @@
           <t>ASTM A36</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1440,7 +1392,6 @@
           <t>ASTM A36</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1477,7 +1428,6 @@
           <t>SAE 1045</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1514,7 +1464,6 @@
           <t>AÇO INOX AISI 420</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1551,7 +1500,6 @@
           <t>ASTM A516 GR70</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1583,8 +1531,6 @@
       <c r="G33" t="n">
         <v>1</v>
       </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1616,8 +1562,6 @@
       <c r="G34" t="n">
         <v>1</v>
       </c>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1649,8 +1593,6 @@
       <c r="G35" t="n">
         <v>1</v>
       </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1728,7 +1670,6 @@
           <t>SAE 8550</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1765,7 +1706,6 @@
           <t>SAE 8550</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1802,7 +1742,6 @@
           <t>ASTM A516 GR70</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1834,8 +1773,6 @@
       <c r="G40" t="n">
         <v>2</v>
       </c>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1867,8 +1804,6 @@
       <c r="G41" t="n">
         <v>2</v>
       </c>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1900,8 +1835,6 @@
       <c r="G42" t="n">
         <v>2</v>
       </c>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1933,8 +1866,6 @@
       <c r="G43" t="n">
         <v>2</v>
       </c>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1966,8 +1897,6 @@
       <c r="G44" t="n">
         <v>2</v>
       </c>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -2004,7 +1933,6 @@
           <t>SAE 8550</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -2041,7 +1969,6 @@
           <t>ASTM A516 GR70</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -2073,8 +2000,6 @@
       <c r="G47" t="n">
         <v>1</v>
       </c>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -2106,8 +2031,6 @@
       <c r="G48" t="n">
         <v>1</v>
       </c>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -2139,8 +2062,6 @@
       <c r="G49" t="n">
         <v>2</v>
       </c>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -2172,8 +2093,6 @@
       <c r="G50" t="n">
         <v>2</v>
       </c>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -2205,8 +2124,6 @@
       <c r="G51" t="n">
         <v>2</v>
       </c>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -2284,7 +2201,6 @@
           <t>SAE 8550</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -2321,7 +2237,6 @@
           <t>ASTM A516 GR70</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -2358,7 +2273,6 @@
           <t>ASTM A36</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -2395,7 +2309,6 @@
           <t>ASTM A516 GR70</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -2432,7 +2345,6 @@
           <t>ASTM A516 GR70</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -2469,7 +2381,6 @@
           <t>ASTM A516 GR70</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -2506,7 +2417,6 @@
           <t>SAE 8550</t>
         </is>
       </c>
-      <c r="I59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -2543,7 +2453,6 @@
           <t>SAE 8550</t>
         </is>
       </c>
-      <c r="I60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -2580,7 +2489,6 @@
           <t>SAE 8550</t>
         </is>
       </c>
-      <c r="I61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -2658,7 +2566,6 @@
           <t>ASTM A36</t>
         </is>
       </c>
-      <c r="I63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -2695,7 +2602,6 @@
           <t>ASTM A36</t>
         </is>
       </c>
-      <c r="I64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -2727,8 +2633,6 @@
       <c r="G65" t="n">
         <v>1</v>
       </c>
-      <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -2760,8 +2664,6 @@
       <c r="G66" t="n">
         <v>1</v>
       </c>
-      <c r="H66" t="inlineStr"/>
-      <c r="I66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -2793,8 +2695,6 @@
       <c r="G67" t="n">
         <v>2</v>
       </c>
-      <c r="H67" t="inlineStr"/>
-      <c r="I67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -2826,8 +2726,6 @@
       <c r="G68" t="n">
         <v>1</v>
       </c>
-      <c r="H68" t="inlineStr"/>
-      <c r="I68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -2840,50 +2738,58 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>03.04.01.3.000598-19-REC</t>
+          <t>03.022-007347-REC</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>BUCHA ESTRIADA</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr"/>
+          <t>CONJUNTO DISCO USINADO</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>022-007347</t>
+        </is>
+      </c>
       <c r="F69" t="n">
         <v>1</v>
       </c>
       <c r="G69" t="n">
         <v>1</v>
       </c>
-      <c r="H69" t="inlineStr"/>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>ASTM A516 GR70</t>
+        </is>
+      </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>Existe no Nomus mas NÃO tem desenho neste PDF — confirmar.</t>
+          <t>Disco existente (REC) 022-007348.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>04.01.3.000598</t>
+          <t>03.022-007347-REC</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>03.022-007347-REC</t>
+          <t>03.022-007346-1</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>CONJUNTO DISCO USINADO</t>
+          <t>CONJUNTO DISCO SOLDADO</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>022-007347</t>
+          <t>022-007346</t>
         </is>
       </c>
       <c r="F70" t="n">
@@ -2891,40 +2797,30 @@
       </c>
       <c r="G70" t="n">
         <v>1</v>
-      </c>
-      <c r="H70" t="inlineStr">
-        <is>
-          <t>ASTM A516 GR70</t>
-        </is>
-      </c>
-      <c r="I70" t="inlineStr">
-        <is>
-          <t>Disco existente (REC) 022-007348.</t>
-        </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>03.022-007347-REC</t>
+          <t>03.022-007346-1</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>03.022-007346-1</t>
+          <t>03.022-007349</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>CONJUNTO DISCO SOLDADO</t>
+          <t>BASE DO DISCO</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>022-007346</t>
+          <t>022-007349</t>
         </is>
       </c>
       <c r="F71" t="n">
@@ -2933,72 +2829,12 @@
       <c r="G71" t="n">
         <v>1</v>
       </c>
-      <c r="H71" t="inlineStr"/>
-      <c r="I71" t="inlineStr"/>
-    </row>
-    <row r="72">
-      <c r="A72" t="n">
-        <v>3</v>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>03.022-007346-1</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>03.022-007349</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>BASE DO DISCO</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>022-007349</t>
-        </is>
-      </c>
-      <c r="F72" t="n">
-        <v>1</v>
-      </c>
-      <c r="G72" t="n">
-        <v>1</v>
-      </c>
-      <c r="H72" t="inlineStr"/>
-      <c r="I72" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="72"/>
     <row r="73">
-      <c r="A73" t="n">
-        <v>1</v>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>04.01.3.000598</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>03.04.01.3.000598-21-REC</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>TAMPA JANELA DE INSPEÇÃO</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr"/>
-      <c r="F73" t="n">
-        <v>1</v>
-      </c>
-      <c r="G73" t="n">
-        <v>1</v>
-      </c>
-      <c r="H73" t="inlineStr"/>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>Existe no Nomus mas NÃO tem desenho neste PDF — confirmar.</t>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>COMPRADOS / NORMALIZADOS (sem código no PDF do Nomus)</t>
         </is>
       </c>
     </row>
@@ -3011,27 +2847,22 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>03.04.01.3.000598-22-REC</t>
-        </is>
-      </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>ATUADOR</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr"/>
+          <t>ROLAM. AUTO-COMPENS. DE ROLOS</t>
+        </is>
+      </c>
       <c r="F74" t="n">
-        <v>1</v>
-      </c>
-      <c r="G74" t="n">
-        <v>1</v>
-      </c>
-      <c r="H74" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>SKF 22312 E Ø60 x Ø130 x 46mm</t>
+        </is>
+      </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>Existe no Nomus mas NÃO tem desenho neste PDF — confirmar.</t>
+          <t>Código Nomus a informar</t>
         </is>
       </c>
     </row>
@@ -3044,36 +2875,78 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>03.04.01.3.000598-23-REC</t>
-        </is>
-      </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>CHAVETA MENOR</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr"/>
+          <t>ANEL ELÁSTICO</t>
+        </is>
+      </c>
       <c r="F75" t="n">
-        <v>1</v>
-      </c>
-      <c r="G75" t="n">
-        <v>1</v>
-      </c>
-      <c r="H75" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>SAE 1070 Ø60 x 2 DIN 471</t>
+        </is>
+      </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>Existe no Nomus mas NÃO tem desenho neste PDF — confirmar.</t>
+          <t>Código Nomus a informar</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>1</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>04.01.3.000598</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>GAXETA QUAD. 2202 TEADIT</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>10</v>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>CARBONO + GRAFITE 3/8" x 3/8" x 3000MM</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Código Nomus a informar</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr"/>
-      <c r="B77" t="inlineStr"/>
-      <c r="C77" s="2" t="inlineStr">
-        <is>
-          <t>COMPRADOS / NORMALIZADOS (sem código no PDF do Nomus)</t>
+      <c r="A77" t="n">
+        <v>1</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>04.01.3.000598</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>PINO ROSCADO M12 x 60</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>4</v>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>CL. 8.8 DIN 976 ZINCADO</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Código Nomus a informar</t>
         </is>
       </c>
     </row>
@@ -3086,20 +2959,17 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr"/>
       <c r="D78" t="inlineStr">
         <is>
-          <t>ROLAM. AUTO-COMPENS. DE ROLOS</t>
-        </is>
-      </c>
-      <c r="E78" t="inlineStr"/>
+          <t>ARRUELA LISA A-13</t>
+        </is>
+      </c>
       <c r="F78" t="n">
-        <v>2</v>
-      </c>
-      <c r="G78" t="inlineStr"/>
+        <v>10</v>
+      </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>SKF 22312 E Ø60 x Ø130 x 46mm</t>
+          <t>CL. 8.8 DIN 125 ZINCADO</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -3117,20 +2987,17 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr"/>
       <c r="D79" t="inlineStr">
         <is>
-          <t>ANEL ELÁSTICO</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr"/>
+          <t>PORCA SEXTAVADA M12</t>
+        </is>
+      </c>
       <c r="F79" t="n">
-        <v>2</v>
-      </c>
-      <c r="G79" t="inlineStr"/>
+        <v>4</v>
+      </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>SAE 1070 Ø60 x 2 DIN 471</t>
+          <t>CL. 8.8 DIN 934 ZINCADO</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -3148,20 +3015,17 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr"/>
       <c r="D80" t="inlineStr">
         <is>
-          <t>GAXETA QUAD. 2202 TEADIT</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr"/>
+          <t>PARAF. CAB. SEXTAVADA M30 x 100</t>
+        </is>
+      </c>
       <c r="F80" t="n">
-        <v>10</v>
-      </c>
-      <c r="G80" t="inlineStr"/>
+        <v>1</v>
+      </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>CARBONO + GRAFITE 3/8" x 3/8" x 3000MM</t>
+          <t>Gr. 8.8 DIN 933</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -3179,20 +3043,17 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr"/>
       <c r="D81" t="inlineStr">
         <is>
-          <t>PINO ROSCADO M12 x 60</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr"/>
+          <t>ARRUELA DE PRESSÃO A-31</t>
+        </is>
+      </c>
       <c r="F81" t="n">
-        <v>4</v>
-      </c>
-      <c r="G81" t="inlineStr"/>
+        <v>2</v>
+      </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>CL. 8.8 DIN 976 ZINCADO</t>
+          <t>DIN 127</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -3210,20 +3071,17 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr"/>
       <c r="D82" t="inlineStr">
         <is>
-          <t>ARRUELA LISA A-13</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr"/>
+          <t>PORCA SEXTAVADA M30</t>
+        </is>
+      </c>
       <c r="F82" t="n">
-        <v>10</v>
-      </c>
-      <c r="G82" t="inlineStr"/>
+        <v>1</v>
+      </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>CL. 8.8 DIN 125 ZINCADO</t>
+          <t>Gr.8 DIN 934</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -3241,20 +3099,17 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr"/>
       <c r="D83" t="inlineStr">
         <is>
-          <t>PORCA SEXTAVADA M12</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr"/>
+          <t>PARAF. CAB. SEXTAVADA M16 x 50</t>
+        </is>
+      </c>
       <c r="F83" t="n">
-        <v>4</v>
-      </c>
-      <c r="G83" t="inlineStr"/>
+        <v>1</v>
+      </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>CL. 8.8 DIN 934 ZINCADO</t>
+          <t>Gr. 8.8 DIN 933</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -3272,20 +3127,17 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr"/>
       <c r="D84" t="inlineStr">
         <is>
-          <t>PARAF. CAB. SEXTAVADA M30 x 100</t>
-        </is>
-      </c>
-      <c r="E84" t="inlineStr"/>
+          <t>PORCA SEXTAVADA M16</t>
+        </is>
+      </c>
       <c r="F84" t="n">
-        <v>1</v>
-      </c>
-      <c r="G84" t="inlineStr"/>
+        <v>17</v>
+      </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Gr. 8.8 DIN 933</t>
+          <t>Gr.8 DIN 934</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -3303,20 +3155,17 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr"/>
       <c r="D85" t="inlineStr">
         <is>
-          <t>ARRUELA DE PRESSÃO A-31</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr"/>
+          <t>ANEL O'RING</t>
+        </is>
+      </c>
       <c r="F85" t="n">
-        <v>2</v>
-      </c>
-      <c r="G85" t="inlineStr"/>
+        <v>1</v>
+      </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>DIN 127</t>
+          <t>VITON FKM 70-75 Sh-A Ø641 x Ø10mm</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -3334,20 +3183,17 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr"/>
       <c r="D86" t="inlineStr">
         <is>
-          <t>PORCA SEXTAVADA M30</t>
-        </is>
-      </c>
-      <c r="E86" t="inlineStr"/>
+          <t>PARAF.ALLEN S/ CAB. SEXT. INTERNO M6 x 25</t>
+        </is>
+      </c>
       <c r="F86" t="n">
-        <v>1</v>
-      </c>
-      <c r="G86" t="inlineStr"/>
+        <v>6</v>
+      </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>Gr.8 DIN 934</t>
+          <t>Gr. 8.8 DIN 913</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -3365,20 +3211,17 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr"/>
       <c r="D87" t="inlineStr">
         <is>
-          <t>PARAF. CAB. SEXTAVADA M16 x 50</t>
-        </is>
-      </c>
-      <c r="E87" t="inlineStr"/>
+          <t>PORCA SEXTAVADA M6</t>
+        </is>
+      </c>
       <c r="F87" t="n">
-        <v>1</v>
-      </c>
-      <c r="G87" t="inlineStr"/>
+        <v>6</v>
+      </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>Gr. 8.8 DIN 933</t>
+          <t>Gr.8 DIN 934</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -3396,17 +3239,14 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr"/>
       <c r="D88" t="inlineStr">
         <is>
-          <t>PORCA SEXTAVADA M16</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr"/>
+          <t>PORCA SEXTAVADA M10</t>
+        </is>
+      </c>
       <c r="F88" t="n">
-        <v>17</v>
-      </c>
-      <c r="G88" t="inlineStr"/>
+        <v>8</v>
+      </c>
       <c r="H88" t="inlineStr">
         <is>
           <t>Gr.8 DIN 934</t>
@@ -3427,20 +3267,17 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr"/>
       <c r="D89" t="inlineStr">
         <is>
-          <t>ANEL O'RING</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr"/>
+          <t>PARAF.ALLEN S/ CAB. SEXT. INTERNO M10 x 40</t>
+        </is>
+      </c>
       <c r="F89" t="n">
-        <v>1</v>
-      </c>
-      <c r="G89" t="inlineStr"/>
+        <v>2</v>
+      </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>VITON FKM 70-75 Sh-A Ø641 x Ø10mm</t>
+          <t>Gr. 8.8 DIN 913</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -3458,20 +3295,17 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr"/>
       <c r="D90" t="inlineStr">
         <is>
-          <t>PARAF.ALLEN S/ CAB. SEXT. INTERNO M6 x 25</t>
-        </is>
-      </c>
-      <c r="E90" t="inlineStr"/>
+          <t>ARRUELA LISA A-10,5</t>
+        </is>
+      </c>
       <c r="F90" t="n">
-        <v>6</v>
-      </c>
-      <c r="G90" t="inlineStr"/>
+        <v>28</v>
+      </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>Gr. 8.8 DIN 913</t>
+          <t>CL. 8.8 DIN 125</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -3489,20 +3323,17 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr"/>
       <c r="D91" t="inlineStr">
         <is>
-          <t>PORCA SEXTAVADA M6</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr"/>
+          <t>PARAF. CAB. SEXTAVADA M10 x 45</t>
+        </is>
+      </c>
       <c r="F91" t="n">
         <v>6</v>
       </c>
-      <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr">
         <is>
-          <t>Gr.8 DIN 934</t>
+          <t>Gr. 8.8 DIN 933</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -3520,20 +3351,17 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr"/>
       <c r="D92" t="inlineStr">
         <is>
-          <t>PORCA SEXTAVADA M10</t>
-        </is>
-      </c>
-      <c r="E92" t="inlineStr"/>
+          <t>PARAF. CAB. SEXTAVADA M12 x 30</t>
+        </is>
+      </c>
       <c r="F92" t="n">
-        <v>8</v>
-      </c>
-      <c r="G92" t="inlineStr"/>
+        <v>6</v>
+      </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>Gr.8 DIN 934</t>
+          <t>Gr. 8.8 DIN 933</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -3551,20 +3379,17 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr"/>
       <c r="D93" t="inlineStr">
         <is>
-          <t>PARAF.ALLEN S/ CAB. SEXT. INTERNO M10 x 40</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr"/>
+          <t>PARAF. CAB. SEXTAVADA M8 x 30</t>
+        </is>
+      </c>
       <c r="F93" t="n">
-        <v>2</v>
-      </c>
-      <c r="G93" t="inlineStr"/>
+        <v>8</v>
+      </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>Gr. 8.8 DIN 913</t>
+          <t>Gr. 8.8 DIN 933</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -3582,20 +3407,17 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C94" t="inlineStr"/>
       <c r="D94" t="inlineStr">
         <is>
-          <t>ARRUELA LISA A-10,5</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr"/>
+          <t>PARAF. CAB. SEXTAVADA M10 x 25</t>
+        </is>
+      </c>
       <c r="F94" t="n">
-        <v>28</v>
-      </c>
-      <c r="G94" t="inlineStr"/>
+        <v>8</v>
+      </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>CL. 8.8 DIN 125</t>
+          <t>Gr. 8.8 DIN 933</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -3613,17 +3435,14 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr"/>
       <c r="D95" t="inlineStr">
         <is>
-          <t>PARAF. CAB. SEXTAVADA M10 x 45</t>
-        </is>
-      </c>
-      <c r="E95" t="inlineStr"/>
+          <t>PARAF. CAB. SEXTAVADA M16 x 45</t>
+        </is>
+      </c>
       <c r="F95" t="n">
-        <v>6</v>
-      </c>
-      <c r="G95" t="inlineStr"/>
+        <v>8</v>
+      </c>
       <c r="H95" t="inlineStr">
         <is>
           <t>Gr. 8.8 DIN 933</t>
@@ -3644,17 +3463,14 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr"/>
       <c r="D96" t="inlineStr">
         <is>
-          <t>PARAF. CAB. SEXTAVADA M12 x 30</t>
-        </is>
-      </c>
-      <c r="E96" t="inlineStr"/>
+          <t>PARAF. CAB. SEXTAVADA M16 x 65</t>
+        </is>
+      </c>
       <c r="F96" t="n">
-        <v>6</v>
-      </c>
-      <c r="G96" t="inlineStr"/>
+        <v>16</v>
+      </c>
       <c r="H96" t="inlineStr">
         <is>
           <t>Gr. 8.8 DIN 933</t>
@@ -3675,20 +3491,17 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr"/>
       <c r="D97" t="inlineStr">
         <is>
-          <t>PARAF. CAB. SEXTAVADA M8 x 30</t>
-        </is>
-      </c>
-      <c r="E97" t="inlineStr"/>
+          <t>NIPLE</t>
+        </is>
+      </c>
       <c r="F97" t="n">
-        <v>8</v>
-      </c>
-      <c r="G97" t="inlineStr"/>
+        <v>10</v>
+      </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>Gr. 8.8 DIN 933</t>
+          <t>AISI 304 1/4" NPT</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -3706,20 +3519,17 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr"/>
       <c r="D98" t="inlineStr">
         <is>
-          <t>PARAF. CAB. SEXTAVADA M10 x 25</t>
-        </is>
-      </c>
-      <c r="E98" t="inlineStr"/>
+          <t>TAMPÃO Ø1" ROSCA BSP ANSI B16.3</t>
+        </is>
+      </c>
       <c r="F98" t="n">
-        <v>8</v>
-      </c>
-      <c r="G98" t="inlineStr"/>
+        <v>2</v>
+      </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>Gr. 8.8 DIN 933</t>
+          <t>ASTM A 197</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -3737,20 +3547,17 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr"/>
       <c r="D99" t="inlineStr">
         <is>
-          <t>PARAF. CAB. SEXTAVADA M16 x 45</t>
-        </is>
-      </c>
-      <c r="E99" t="inlineStr"/>
+          <t>UNIÃO ORIENTÁVEL SIMPLES</t>
+        </is>
+      </c>
       <c r="F99" t="n">
-        <v>8</v>
-      </c>
-      <c r="G99" t="inlineStr"/>
+        <v>2</v>
+      </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>Gr. 8.8 DIN 933</t>
+          <t>AISI 304 1/4" NPT</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -3768,20 +3575,17 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C100" t="inlineStr"/>
       <c r="D100" t="inlineStr">
         <is>
-          <t>PARAF. CAB. SEXTAVADA M16 x 65</t>
-        </is>
-      </c>
-      <c r="E100" t="inlineStr"/>
+          <t>DISTRIBUIDOR LINHA DUPLA BM-4</t>
+        </is>
+      </c>
       <c r="F100" t="n">
-        <v>16</v>
-      </c>
-      <c r="G100" t="inlineStr"/>
+        <v>1</v>
+      </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>Gr. 8.8 DIN 933</t>
+          <t>04 MÓDULOS/08 SAÍDAS EXIMPORT</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -3799,20 +3603,17 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr"/>
       <c r="D101" t="inlineStr">
         <is>
-          <t>NIPLE</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr"/>
+          <t>ARRUELA LISA A-8,1</t>
+        </is>
+      </c>
       <c r="F101" t="n">
-        <v>10</v>
-      </c>
-      <c r="G101" t="inlineStr"/>
+        <v>2</v>
+      </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>AISI 304 1/4" NPT</t>
+          <t>CL. 8.8 DIN 125</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -3830,20 +3631,17 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr"/>
       <c r="D102" t="inlineStr">
         <is>
-          <t>TAMPÃO Ø1" ROSCA BSP ANSI B16.3</t>
-        </is>
-      </c>
-      <c r="E102" t="inlineStr"/>
+          <t>PORCA SEXTAVADA M10</t>
+        </is>
+      </c>
       <c r="F102" t="n">
         <v>2</v>
       </c>
-      <c r="G102" t="inlineStr"/>
       <c r="H102" t="inlineStr">
         <is>
-          <t>ASTM A 197</t>
+          <t>Gr.8 DIN 934</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -3861,17 +3659,14 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C103" t="inlineStr"/>
       <c r="D103" t="inlineStr">
         <is>
-          <t>UNIÃO ORIENTÁVEL SIMPLES</t>
-        </is>
-      </c>
-      <c r="E103" t="inlineStr"/>
+          <t>TÊ ROSCA FÊMEA 6000Lbs</t>
+        </is>
+      </c>
       <c r="F103" t="n">
-        <v>2</v>
-      </c>
-      <c r="G103" t="inlineStr"/>
+        <v>4</v>
+      </c>
       <c r="H103" t="inlineStr">
         <is>
           <t>AISI 304 1/4" NPT</t>
@@ -3892,20 +3687,17 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C104" t="inlineStr"/>
       <c r="D104" t="inlineStr">
         <is>
-          <t>DISTRIBUIDOR LINHA DUPLA BM-4</t>
-        </is>
-      </c>
-      <c r="E104" t="inlineStr"/>
+          <t>TUBO Ø10 PAREDE 1MM X 6000MM</t>
+        </is>
+      </c>
       <c r="F104" t="n">
         <v>1</v>
       </c>
-      <c r="G104" t="inlineStr"/>
       <c r="H104" t="inlineStr">
         <is>
-          <t>04 MÓDULOS/08 SAÍDAS EXIMPORT</t>
+          <t>AISI 304</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -3923,20 +3715,17 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr"/>
       <c r="D105" t="inlineStr">
         <is>
-          <t>ARRUELA LISA A-8,1</t>
-        </is>
-      </c>
-      <c r="E105" t="inlineStr"/>
+          <t>CONEXÃO JOELHO PARA TUBO 10MM</t>
+        </is>
+      </c>
       <c r="F105" t="n">
         <v>2</v>
       </c>
-      <c r="G105" t="inlineStr"/>
       <c r="H105" t="inlineStr">
         <is>
-          <t>CL. 8.8 DIN 125</t>
+          <t>AISI 304 1/4" NPT</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -3954,20 +3743,17 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C106" t="inlineStr"/>
       <c r="D106" t="inlineStr">
         <is>
-          <t>PORCA SEXTAVADA M10</t>
-        </is>
-      </c>
-      <c r="E106" t="inlineStr"/>
+          <t>PARAF.ALLEN C/CAB.SEXT. INTER. M6 x 55</t>
+        </is>
+      </c>
       <c r="F106" t="n">
         <v>2</v>
       </c>
-      <c r="G106" t="inlineStr"/>
       <c r="H106" t="inlineStr">
         <is>
-          <t>Gr.8 DIN 934</t>
+          <t>Gr. 8.8 DIN 912</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -3985,20 +3771,17 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr"/>
       <c r="D107" t="inlineStr">
         <is>
-          <t>TÊ ROSCA FÊMEA 6000Lbs</t>
-        </is>
-      </c>
-      <c r="E107" t="inlineStr"/>
+          <t>GAXETA QUAD. 2202 TEADIT</t>
+        </is>
+      </c>
       <c r="F107" t="n">
-        <v>4</v>
-      </c>
-      <c r="G107" t="inlineStr"/>
+        <v>1</v>
+      </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>AISI 304 1/4" NPT</t>
+          <t>CARBONO + GRAFITE 1/4" x 1/4" x 900MM</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -4016,25 +3799,27 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C108" t="inlineStr"/>
       <c r="D108" t="inlineStr">
         <is>
-          <t>TUBO Ø10 PAREDE 1MM X 6000MM</t>
-        </is>
-      </c>
-      <c r="E108" t="inlineStr"/>
+          <t>JUNTA METALBEST (022-007370)</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>022-007370</t>
+        </is>
+      </c>
       <c r="F108" t="n">
-        <v>1</v>
-      </c>
-      <c r="G108" t="inlineStr"/>
+        <v>2</v>
+      </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>AISI 304</t>
+          <t>INOX / GRAFITE</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>Código Nomus a informar</t>
+          <t>Comprado — código Nomus a informar</t>
         </is>
       </c>
     </row>
@@ -4047,145 +3832,12 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="C109" t="inlineStr"/>
       <c r="D109" t="inlineStr">
         <is>
-          <t>CONEXÃO JOELHO PARA TUBO 10MM</t>
-        </is>
-      </c>
-      <c r="E109" t="inlineStr"/>
-      <c r="F109" t="n">
-        <v>2</v>
-      </c>
-      <c r="G109" t="inlineStr"/>
-      <c r="H109" t="inlineStr">
-        <is>
-          <t>AISI 304 1/4" NPT</t>
+          <t>PENDENTE: balões 52, 62, 65 sem linha na lista do desenho</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
-        <is>
-          <t>Código Nomus a informar</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="n">
-        <v>1</v>
-      </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>04.01.3.000598</t>
-        </is>
-      </c>
-      <c r="C110" t="inlineStr"/>
-      <c r="D110" t="inlineStr">
-        <is>
-          <t>PARAF.ALLEN C/CAB.SEXT. INTER. M6 x 55</t>
-        </is>
-      </c>
-      <c r="E110" t="inlineStr"/>
-      <c r="F110" t="n">
-        <v>2</v>
-      </c>
-      <c r="G110" t="inlineStr"/>
-      <c r="H110" t="inlineStr">
-        <is>
-          <t>Gr. 8.8 DIN 912</t>
-        </is>
-      </c>
-      <c r="I110" t="inlineStr">
-        <is>
-          <t>Código Nomus a informar</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="n">
-        <v>1</v>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>04.01.3.000598</t>
-        </is>
-      </c>
-      <c r="C111" t="inlineStr"/>
-      <c r="D111" t="inlineStr">
-        <is>
-          <t>GAXETA QUAD. 2202 TEADIT</t>
-        </is>
-      </c>
-      <c r="E111" t="inlineStr"/>
-      <c r="F111" t="n">
-        <v>1</v>
-      </c>
-      <c r="G111" t="inlineStr"/>
-      <c r="H111" t="inlineStr">
-        <is>
-          <t>CARBONO + GRAFITE 1/4" x 1/4" x 900MM</t>
-        </is>
-      </c>
-      <c r="I111" t="inlineStr">
-        <is>
-          <t>Código Nomus a informar</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="n">
-        <v>1</v>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>04.01.3.000598</t>
-        </is>
-      </c>
-      <c r="C112" t="inlineStr"/>
-      <c r="D112" t="inlineStr">
-        <is>
-          <t>JUNTA METALBEST (022-007370)</t>
-        </is>
-      </c>
-      <c r="E112" t="inlineStr">
-        <is>
-          <t>022-007370</t>
-        </is>
-      </c>
-      <c r="F112" t="n">
-        <v>2</v>
-      </c>
-      <c r="G112" t="inlineStr"/>
-      <c r="H112" t="inlineStr">
-        <is>
-          <t>INOX / GRAFITE</t>
-        </is>
-      </c>
-      <c r="I112" t="inlineStr">
-        <is>
-          <t>Comprado — código Nomus a informar</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="n">
-        <v>1</v>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>04.01.3.000598</t>
-        </is>
-      </c>
-      <c r="C113" t="inlineStr"/>
-      <c r="D113" t="inlineStr">
-        <is>
-          <t>PENDENTE: balões 52, 62, 65 sem linha na lista do desenho</t>
-        </is>
-      </c>
-      <c r="E113" t="inlineStr"/>
-      <c r="F113" t="inlineStr"/>
-      <c r="G113" t="inlineStr"/>
-      <c r="H113" t="inlineStr"/>
-      <c r="I113" t="inlineStr">
         <is>
           <t>Definir descrição, material e qtd</t>
         </is>

</xml_diff>

<commit_message>
Add raw-material columns to each part row
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019oxoH766RXuqLqXQEjeJHj
</commit_message>
<xml_diff>
--- a/Estrutura_04.01.3.000598.xlsx
+++ b/Estrutura_04.01.3.000598.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A conferir" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Importação'!$A$1:$G$160</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Importação'!$A$1:$K$160</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,50 +440,74 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G160"/>
+  <dimension ref="A1:K160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="80" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="70" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Código pai</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Código do componente</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Descrição</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Qtd</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Un</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Matéria-prima (código)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Matéria-prima (descrição)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Qtd matéria-prima</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Un MP</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Observação</t>
         </is>
@@ -518,7 +542,11 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
         <is>
           <t>Corpo existente (REC).</t>
         </is>
@@ -554,6 +582,9 @@
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -584,7 +615,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>01.13.1.57.14.24</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>TUBO Ø175 x Ø150 ASTM A516 Gr 70 .</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>125</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -617,6 +665,24 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
+          <t>01.13.1.57.14.24</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>TUBO Ø175 x Ø150 ASTM A516 Gr 70 .</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>125</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
           <t xml:space="preserve">(mm) </t>
         </is>
       </c>
@@ -650,7 +716,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>01.09.3.1.2.4.6</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 516 Gr 70 1"</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -683,6 +766,24 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
+          <t>01.09.3.1.2.4.6</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 516 Gr 70 1"</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
           <t xml:space="preserve">(kg bruto calculado) </t>
         </is>
       </c>
@@ -716,7 +817,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>01.09.1.1.36.1.78</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>BARRA REDONDA 5" AÇO CARBONO ASTM A516 Gr.70</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>125</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -749,6 +867,24 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
+          <t>01.09.1.1.36.1.78</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>BARRA REDONDA 5" AÇO CARBONO ASTM A516 Gr.70</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>125</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
           <t xml:space="preserve">(mm) </t>
         </is>
       </c>
@@ -782,7 +918,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>01.09.1.1.12.1.78</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>BARRA REDONDA 1 1/4" AÇO CARBONO ASTM A516 Gr.70</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>55</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -815,6 +968,24 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
+          <t>01.09.1.1.12.1.78</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>BARRA REDONDA 1 1/4" AÇO CARBONO ASTM A516 Gr.70</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>55</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
           <t xml:space="preserve">(mm) </t>
         </is>
       </c>
@@ -849,6 +1020,9 @@
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -880,6 +1054,9 @@
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -910,7 +1087,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>01.09.3.1.2.4.3</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 516 Gr 70 5/8"</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -943,6 +1137,24 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
+          <t>01.09.3.1.2.4.3</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 516 Gr 70 5/8"</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
           <t xml:space="preserve">(kg bruto calculado) </t>
         </is>
       </c>
@@ -976,7 +1188,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>01.09.3.1.2.4.4</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 516 Gr 70 3/4"</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1009,6 +1238,24 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
+          <t>01.09.3.1.2.4.4</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 516 Gr 70 3/4"</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
           <t xml:space="preserve">(kg bruto calculado) </t>
         </is>
       </c>
@@ -1043,6 +1290,9 @@
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1073,7 +1323,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>01.09.3.1.1.5.52</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 36 - 1"</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>12.46</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1106,6 +1373,24 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
+          <t>01.09.3.1.1.5.52</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 36 - 1"</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>12.46</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
           <t xml:space="preserve">(kg bruto calculado) </t>
         </is>
       </c>
@@ -1139,7 +1424,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>01.09.3.1.1.5.3</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 36 - 5/8"</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>3.07</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1172,6 +1474,24 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
+          <t>01.09.3.1.1.5.3</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 36 - 5/8"</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>3.07</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
           <t xml:space="preserve">(kg bruto calculado) </t>
         </is>
       </c>
@@ -1205,7 +1525,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>01.09.3.1.1.5.3</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 36 - 5/8"</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>5.88</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1238,6 +1575,24 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
+          <t>01.09.3.1.1.5.3</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 36 - 5/8"</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>5.88</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
           <t xml:space="preserve">(kg bruto calculado) </t>
         </is>
       </c>
@@ -1271,7 +1626,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>01.09.3.1.1.5.3</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 36 - 5/8"</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1304,6 +1676,24 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
+          <t>01.09.3.1.1.5.3</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 36 - 5/8"</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
           <t xml:space="preserve">(kg bruto calculado) </t>
         </is>
       </c>
@@ -1337,7 +1727,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>01.09.3.1.1.5.3</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 36 - 5/8"</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1370,6 +1777,24 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
+          <t>01.09.3.1.1.5.3</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 36 - 5/8"</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
           <t xml:space="preserve">(kg bruto calculado) </t>
         </is>
       </c>
@@ -1403,7 +1828,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>01.09.3.1.1.5.19</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 36 - 1/8"</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1436,6 +1878,24 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
+          <t>01.09.3.1.1.5.19</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 36 - 1/8"</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
           <t xml:space="preserve">(kg bruto calculado) </t>
         </is>
       </c>
@@ -1469,7 +1929,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>01.09.3.1.2.4.11</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 516 Gr 70 1/2"</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1502,6 +1979,24 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
+          <t>01.09.3.1.2.4.11</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 516 Gr 70 1/2"</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
           <t xml:space="preserve">(kg bruto calculado) </t>
         </is>
       </c>
@@ -1535,7 +2030,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>01.09.1.1.30.3.1</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>BARRA REDONDA 3 1/2" AÇO INOX AISI 304</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>20</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1568,6 +2080,24 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
+          <t>01.09.1.1.30.3.1</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>BARRA REDONDA 3 1/2" AÇO INOX AISI 304</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>20</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
           <t xml:space="preserve">(mm) </t>
         </is>
       </c>
@@ -1601,7 +2131,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>01.09.1.1.30.3.1</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>BARRA REDONDA 3 1/2" AÇO INOX AISI 304</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>15</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1634,6 +2181,24 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
+          <t>01.09.1.1.30.3.1</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>BARRA REDONDA 3 1/2" AÇO INOX AISI 304</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>15</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
           <t xml:space="preserve">(mm) </t>
         </is>
       </c>
@@ -1668,6 +2233,9 @@
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1699,6 +2267,9 @@
         </is>
       </c>
       <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1729,7 +2300,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>01.09.3.1.2.4.6</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 516 Gr 70 1"</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>15.08</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1762,6 +2350,24 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
+          <t>01.09.3.1.2.4.6</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 516 Gr 70 1"</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>15.08</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
           <t xml:space="preserve">(kg bruto calculado) </t>
         </is>
       </c>
@@ -1795,7 +2401,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>01.13.1.5.4.4</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>TUBO 1" ASTM A36 SCH 80</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>50</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1828,6 +2451,24 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
+          <t>01.13.1.5.4.4</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>TUBO 1" ASTM A36 SCH 80</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>50</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
           <t xml:space="preserve">(mm) </t>
         </is>
       </c>
@@ -1861,7 +2502,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>01.09.3.1.1.5.11</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 36 - 1/2"</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1894,6 +2552,24 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
+          <t>01.09.3.1.1.5.11</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 36 - 1/2"</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
           <t xml:space="preserve">(kg bruto calculado) </t>
         </is>
       </c>
@@ -1927,7 +2603,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr"/>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>01.09.3.1.1.5.4</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 36 - 3/4"</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1960,6 +2653,24 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
+          <t>01.09.3.1.1.5.4</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 36 - 3/4"</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
           <t xml:space="preserve">(kg bruto calculado) </t>
         </is>
       </c>
@@ -1993,7 +2704,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr"/>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>01.09.3.1.1.5.3</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 36 - 5/8"</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2026,6 +2754,24 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
+          <t>01.09.3.1.1.5.3</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 36 - 5/8"</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
           <t xml:space="preserve">(kg bruto calculado) </t>
         </is>
       </c>
@@ -2059,7 +2805,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr"/>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>01.09.1.10.224.1.22</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>BARRA CHAVETA 17 x 25 AÇO CARBONO SAE 1045</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>155</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2092,6 +2855,24 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
+          <t>01.09.1.10.224.1.22</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>BARRA CHAVETA 17 x 25 AÇO CARBONO SAE 1045</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>155</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
           <t xml:space="preserve">(mm) </t>
         </is>
       </c>
@@ -2125,7 +2906,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr"/>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>01.09.1.1.27.3.7</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>BARRA REDONDA 3" AÇO INOX AISI 420</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>1250</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2158,6 +2956,24 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
+          <t>01.09.1.1.27.3.7</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>BARRA REDONDA 3" AÇO INOX AISI 420</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>1250</v>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
           <t xml:space="preserve">(mm) </t>
         </is>
       </c>
@@ -2192,6 +3008,9 @@
         </is>
       </c>
       <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2223,6 +3042,9 @@
         </is>
       </c>
       <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2253,7 +3075,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr"/>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>01.09.3.1.2.4.6</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 516 Gr 70 1"</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>11.95</v>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2286,6 +3125,24 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
+          <t>01.09.3.1.2.4.6</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 516 Gr 70 1"</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>11.95</v>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
           <t xml:space="preserve">(kg bruto calculado) </t>
         </is>
       </c>
@@ -2319,7 +3176,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr"/>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>01.13.1.58.12.24</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>TUBO Ø50 x Ø27 SAE 8550 .</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>38</v>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2352,6 +3226,24 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
+          <t>01.13.1.58.12.24</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>TUBO Ø50 x Ø27 SAE 8550 .</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>38</v>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
           <t xml:space="preserve">(mm) </t>
         </is>
       </c>
@@ -2387,6 +3279,24 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
+          <t>01.09.1.1.1.1.9</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>BARRA REDONDA 1/4" AÇO CARBONO SAE 1020</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>10</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
           <t>Matéria-prima Ø6 x 10 mm (sobremetal).</t>
         </is>
       </c>
@@ -2422,6 +3332,24 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
+          <t>01.09.1.1.1.1.9</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>BARRA REDONDA 1/4" AÇO CARBONO SAE 1020</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>10</v>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
           <t>(mm) Ø6 x 10 mm (sobremetal de usinagem, decisão).</t>
         </is>
       </c>
@@ -2455,7 +3383,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr"/>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>01.13.1.59.12.24</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>TUBO Ø110 x Ø90 SAE 8550 .</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>30</v>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2488,6 +3433,24 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
+          <t>01.13.1.59.12.24</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>TUBO Ø110 x Ø90 SAE 8550 .</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
+        <v>30</v>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
           <t xml:space="preserve">(mm) </t>
         </is>
       </c>
@@ -2521,7 +3484,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G63" t="inlineStr"/>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>01.13.1.60.12.24</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>TUBO Ø105 x Ø60 SAE 8550 .</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
+        <v>35</v>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2554,6 +3534,24 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
+          <t>01.13.1.60.12.24</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>TUBO Ø105 x Ø60 SAE 8550 .</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
+        <v>35</v>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
           <t xml:space="preserve">(mm) </t>
         </is>
       </c>
@@ -2588,6 +3586,9 @@
         </is>
       </c>
       <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2619,6 +3620,9 @@
         </is>
       </c>
       <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2649,7 +3653,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr"/>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>01.13.1.61.1.24</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>TUBO Ø4" x Ø60 ASTM A106 GR C .</t>
+        </is>
+      </c>
+      <c r="I67" t="n">
+        <v>90</v>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2682,6 +3703,24 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
+          <t>01.13.1.61.1.24</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>TUBO Ø4" x Ø60 ASTM A106 GR C .</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
+        <v>90</v>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
           <t xml:space="preserve">(mm) </t>
         </is>
       </c>
@@ -2715,7 +3754,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr"/>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>01.09.3.1.2.4.3</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 516 Gr 70 5/8"</t>
+        </is>
+      </c>
+      <c r="I69" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2748,6 +3804,24 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
+          <t>01.09.3.1.2.4.3</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 516 Gr 70 5/8"</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
           <t xml:space="preserve">(kg bruto calculado) </t>
         </is>
       </c>
@@ -2782,6 +3856,9 @@
         </is>
       </c>
       <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
@@ -2789,20 +3866,24 @@
           <t>03.022-007345</t>
         </is>
       </c>
-      <c r="B72" s="4" t="inlineStr"/>
+      <c r="B72" s="4" t="n"/>
       <c r="C72" s="4" t="inlineStr">
         <is>
           <t>[DEFINIR] Matéria-prima da barra superior da alavanca (sem desenho 022-007345)</t>
         </is>
       </c>
-      <c r="D72" s="4" t="inlineStr"/>
-      <c r="E72" s="4" t="inlineStr"/>
+      <c r="D72" s="4" t="n"/>
+      <c r="E72" s="4" t="n"/>
       <c r="F72" s="4" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="G72" s="4" t="inlineStr">
+      <c r="G72" s="4" t="inlineStr"/>
+      <c r="H72" s="4" t="inlineStr"/>
+      <c r="I72" s="4" t="inlineStr"/>
+      <c r="J72" s="4" t="inlineStr"/>
+      <c r="K72" s="4" t="inlineStr">
         <is>
           <t>Sem desenho no PDF; peça espelhada da barra inferior (007350, chapa 1/2" A516 Gr70)?</t>
         </is>
@@ -2837,7 +3918,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr"/>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>01.09.3.1.2.4.11</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 516 Gr 70 1/2"</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2870,6 +3968,24 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
+          <t>01.09.3.1.2.4.11</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 516 Gr 70 1/2"</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
           <t xml:space="preserve">(kg bruto calculado) </t>
         </is>
       </c>
@@ -2903,7 +4019,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>01.13.1.62.12.24</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>TUBO Ø35 x Ø55 SAE 8550 .</t>
+        </is>
+      </c>
+      <c r="I75" t="n">
+        <v>20</v>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2936,6 +4069,24 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
+          <t>01.13.1.62.12.24</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>TUBO Ø35 x Ø55 SAE 8550 .</t>
+        </is>
+      </c>
+      <c r="I76" t="n">
+        <v>20</v>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
           <t xml:space="preserve">(mm) </t>
         </is>
       </c>
@@ -2970,6 +4121,9 @@
         </is>
       </c>
       <c r="G77" t="inlineStr"/>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr"/>
+      <c r="J77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3001,6 +4155,9 @@
         </is>
       </c>
       <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr"/>
+      <c r="J78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3031,7 +4188,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G79" t="inlineStr"/>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>01.09.3.1.2.4.11</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 516 Gr 70 1/2"</t>
+        </is>
+      </c>
+      <c r="I79" t="n">
+        <v>2.83</v>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3064,6 +4238,24 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
+          <t>01.09.3.1.2.4.11</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 516 Gr 70 1/2"</t>
+        </is>
+      </c>
+      <c r="I80" t="n">
+        <v>2.83</v>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
           <t xml:space="preserve">(kg bruto calculado) </t>
         </is>
       </c>
@@ -3097,7 +4289,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G81" t="inlineStr"/>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>01.09.3.1.2.4.3</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 516 Gr 70 5/8"</t>
+        </is>
+      </c>
+      <c r="I81" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -3130,6 +4339,24 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
+          <t>01.09.3.1.2.4.3</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 516 Gr 70 5/8"</t>
+        </is>
+      </c>
+      <c r="I82" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
           <t xml:space="preserve">(kg bruto calculado) </t>
         </is>
       </c>
@@ -3163,7 +4390,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G83" t="inlineStr"/>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>01.13.1.63.12.24</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>TUBO Ø60 x Ø30 SAE 8550 .</t>
+        </is>
+      </c>
+      <c r="I83" t="n">
+        <v>25</v>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3196,6 +4440,24 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
+          <t>01.13.1.63.12.24</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>TUBO Ø60 x Ø30 SAE 8550 .</t>
+        </is>
+      </c>
+      <c r="I84" t="n">
+        <v>25</v>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
           <t xml:space="preserve">(mm) </t>
         </is>
       </c>
@@ -3229,7 +4491,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G85" t="inlineStr"/>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>01.13.1.58.12.24</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>TUBO Ø50 x Ø27 SAE 8550 .</t>
+        </is>
+      </c>
+      <c r="I85" t="n">
+        <v>25</v>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -3262,6 +4541,24 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
+          <t>01.13.1.58.12.24</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>TUBO Ø50 x Ø27 SAE 8550 .</t>
+        </is>
+      </c>
+      <c r="I86" t="n">
+        <v>25</v>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
           <t xml:space="preserve">(mm) </t>
         </is>
       </c>
@@ -3297,6 +4594,24 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
+          <t>01.09.1.1.1.1.9</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>BARRA REDONDA 1/4" AÇO CARBONO SAE 1020</t>
+        </is>
+      </c>
+      <c r="I87" t="n">
+        <v>10</v>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
           <t>Matéria-prima Ø6 x 10 mm (sobremetal).</t>
         </is>
       </c>
@@ -3332,6 +4647,24 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
+          <t>01.09.1.1.1.1.9</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>BARRA REDONDA 1/4" AÇO CARBONO SAE 1020</t>
+        </is>
+      </c>
+      <c r="I88" t="n">
+        <v>10</v>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
           <t>(mm) Ø6 x 10 mm (sobremetal de usinagem, decisão).</t>
         </is>
       </c>
@@ -3365,7 +4698,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G89" t="inlineStr"/>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>01.13.1.58.12.24</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>TUBO Ø50 x Ø27 SAE 8550 .</t>
+        </is>
+      </c>
+      <c r="I89" t="n">
+        <v>20</v>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -3398,6 +4748,24 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
+          <t>01.13.1.58.12.24</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>TUBO Ø50 x Ø27 SAE 8550 .</t>
+        </is>
+      </c>
+      <c r="I90" t="n">
+        <v>20</v>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
           <t xml:space="preserve">(mm) </t>
         </is>
       </c>
@@ -3431,7 +4799,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G91" t="inlineStr"/>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>01.09.3.1.2.4.3</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 516 Gr 70 5/8"</t>
+        </is>
+      </c>
+      <c r="I91" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3464,6 +4849,24 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
+          <t>01.09.3.1.2.4.3</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 516 Gr 70 5/8"</t>
+        </is>
+      </c>
+      <c r="I92" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
           <t xml:space="preserve">(kg bruto calculado) </t>
         </is>
       </c>
@@ -3497,7 +4900,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G93" t="inlineStr"/>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>01.09.1.1.44.1.9</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>BARRA REDONDA 7" AÇO CARBONO SAE 1020</t>
+        </is>
+      </c>
+      <c r="I93" t="n">
+        <v>70</v>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -3530,6 +4950,24 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
+          <t>01.09.1.1.44.1.9</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>BARRA REDONDA 7" AÇO CARBONO SAE 1020</t>
+        </is>
+      </c>
+      <c r="I94" t="n">
+        <v>70</v>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
           <t>(mm) CONFERIR: desenho pede ASTM A36 Ø7"; no cadastro só existe Ø7" SAE 1020 (não há A36).</t>
         </is>
       </c>
@@ -3563,7 +5001,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G95" t="inlineStr"/>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>01.09.3.1.2.4.11</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 516 Gr 70 1/2"</t>
+        </is>
+      </c>
+      <c r="I95" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -3596,6 +5051,24 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
+          <t>01.09.3.1.2.4.11</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 516 Gr 70 1/2"</t>
+        </is>
+      </c>
+      <c r="I96" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
           <t xml:space="preserve">(kg bruto calculado) </t>
         </is>
       </c>
@@ -3629,7 +5102,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G97" t="inlineStr"/>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>01.09.3.1.2.4.6</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 516 Gr 70 1"</t>
+        </is>
+      </c>
+      <c r="I97" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -3662,6 +5152,24 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
+          <t>01.09.3.1.2.4.6</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 516 Gr 70 1"</t>
+        </is>
+      </c>
+      <c r="I98" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
           <t xml:space="preserve">(kg bruto calculado) </t>
         </is>
       </c>
@@ -3695,7 +5203,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G99" t="inlineStr"/>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>01.09.3.1.2.4.11</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 516 Gr 70 1/2"</t>
+        </is>
+      </c>
+      <c r="I99" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -3728,6 +5253,24 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
+          <t>01.09.3.1.2.4.11</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 516 Gr 70 1/2"</t>
+        </is>
+      </c>
+      <c r="I100" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
           <t xml:space="preserve">(kg bruto calculado) </t>
         </is>
       </c>
@@ -3761,7 +5304,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G101" t="inlineStr"/>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>01.09.1.1.17.1.27</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>BARRA REDONDA 1 3/4" AÇO CARBONO SAE 8550</t>
+        </is>
+      </c>
+      <c r="I101" t="n">
+        <v>160</v>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -3794,6 +5354,24 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
+          <t>01.09.1.1.17.1.27</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>BARRA REDONDA 1 3/4" AÇO CARBONO SAE 8550</t>
+        </is>
+      </c>
+      <c r="I102" t="n">
+        <v>160</v>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
           <t xml:space="preserve">(mm) </t>
         </is>
       </c>
@@ -3827,7 +5405,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G103" t="inlineStr"/>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>01.09.1.1.15.1.27</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>BARRA REDONDA 1 1/2" AÇO CARBONO SAE 8550</t>
+        </is>
+      </c>
+      <c r="I103" t="n">
+        <v>100</v>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -3860,6 +5455,24 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
+          <t>01.09.1.1.15.1.27</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>BARRA REDONDA 1 1/2" AÇO CARBONO SAE 8550</t>
+        </is>
+      </c>
+      <c r="I104" t="n">
+        <v>100</v>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
           <t xml:space="preserve">(mm) </t>
         </is>
       </c>
@@ -3893,7 +5506,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G105" t="inlineStr"/>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>01.09.1.1.15.1.27</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>BARRA REDONDA 1 1/2" AÇO CARBONO SAE 8550</t>
+        </is>
+      </c>
+      <c r="I105" t="n">
+        <v>120</v>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -3926,6 +5556,24 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
+          <t>01.09.1.1.15.1.27</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>BARRA REDONDA 1 1/2" AÇO CARBONO SAE 8550</t>
+        </is>
+      </c>
+      <c r="I106" t="n">
+        <v>120</v>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
           <t xml:space="preserve">(mm) </t>
         </is>
       </c>
@@ -3961,6 +5609,24 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
+          <t>01.09.1.1.1.1.9</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>BARRA REDONDA 1/4" AÇO CARBONO SAE 1020</t>
+        </is>
+      </c>
+      <c r="I107" t="n">
+        <v>10</v>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
           <t>Matéria-prima Ø6 x 10 mm (sobremetal).</t>
         </is>
       </c>
@@ -3996,6 +5662,24 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
+          <t>01.09.1.1.1.1.9</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>BARRA REDONDA 1/4" AÇO CARBONO SAE 1020</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
+        <v>10</v>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>MILIMETRO</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
           <t>(mm) Ø6 x 10 mm (sobremetal de usinagem, decisão).</t>
         </is>
       </c>
@@ -4029,7 +5713,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G109" t="inlineStr"/>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>01.09.3.1.1.5.3</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 36 - 5/8"</t>
+        </is>
+      </c>
+      <c r="I109" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -4062,6 +5763,24 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
+          <t>01.09.3.1.1.5.3</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 36 - 5/8"</t>
+        </is>
+      </c>
+      <c r="I110" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
           <t xml:space="preserve">(kg bruto calculado) </t>
         </is>
       </c>
@@ -4096,6 +5815,9 @@
         </is>
       </c>
       <c r="G111" t="inlineStr"/>
+      <c r="H111" t="inlineStr"/>
+      <c r="I111" t="inlineStr"/>
+      <c r="J111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -4127,6 +5849,9 @@
         </is>
       </c>
       <c r="G112" t="inlineStr"/>
+      <c r="H112" t="inlineStr"/>
+      <c r="I112" t="inlineStr"/>
+      <c r="J112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -4157,7 +5882,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G113" t="inlineStr"/>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>01.09.3.1.1.5.4</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 36 - 3/4"</t>
+        </is>
+      </c>
+      <c r="I113" t="n">
+        <v>9.35</v>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -4190,6 +5932,24 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
+          <t>01.09.3.1.1.5.4</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 36 - 3/4"</t>
+        </is>
+      </c>
+      <c r="I114" t="n">
+        <v>9.35</v>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
           <t>(kg bruto calculado) Espessura 3/4" (decisão).</t>
         </is>
       </c>
@@ -4223,7 +5983,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G115" t="inlineStr"/>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>01.09.3.1.1.5.3</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 36 - 5/8"</t>
+        </is>
+      </c>
+      <c r="I115" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -4256,6 +6033,24 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
+          <t>01.09.3.1.1.5.3</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 36 - 5/8"</t>
+        </is>
+      </c>
+      <c r="I116" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
           <t xml:space="preserve">(kg bruto calculado) </t>
         </is>
       </c>
@@ -4289,7 +6084,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G117" t="inlineStr"/>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>01.09.3.1.1.5.4</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 36 - 3/4"</t>
+        </is>
+      </c>
+      <c r="I117" t="n">
+        <v>9.35</v>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -4322,6 +6134,24 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
+          <t>01.09.3.1.1.5.4</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 36 - 3/4"</t>
+        </is>
+      </c>
+      <c r="I118" t="n">
+        <v>9.35</v>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
           <t xml:space="preserve">(kg bruto calculado) </t>
         </is>
       </c>
@@ -4355,7 +6185,11 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G119" t="inlineStr">
+      <c r="G119" t="inlineStr"/>
+      <c r="H119" t="inlineStr"/>
+      <c r="I119" t="inlineStr"/>
+      <c r="J119" t="inlineStr"/>
+      <c r="K119" t="inlineStr">
         <is>
           <t>Disco existente (REC) 022-007348.</t>
         </is>
@@ -4391,6 +6225,9 @@
         </is>
       </c>
       <c r="G120" t="inlineStr"/>
+      <c r="H120" t="inlineStr"/>
+      <c r="I120" t="inlineStr"/>
+      <c r="J120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -4421,7 +6258,24 @@
           <t>Fabricado</t>
         </is>
       </c>
-      <c r="G121" t="inlineStr"/>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>01.09.3.1.2.4.3</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 516 Gr 70 5/8"</t>
+        </is>
+      </c>
+      <c r="I121" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -4454,6 +6308,24 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
+          <t>01.09.3.1.2.4.3</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>CHAPA LISA AÇO CARBONO - ASTM A 516 Gr 70 5/8"</t>
+        </is>
+      </c>
+      <c r="I122" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>QUILOGRAMA</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
           <t xml:space="preserve">(kg bruto calculado) </t>
         </is>
       </c>
@@ -4488,6 +6360,9 @@
         </is>
       </c>
       <c r="G123" t="inlineStr"/>
+      <c r="H123" t="inlineStr"/>
+      <c r="I123" t="inlineStr"/>
+      <c r="J123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -4518,7 +6393,11 @@
           <t>Comprado</t>
         </is>
       </c>
-      <c r="G124" t="inlineStr">
+      <c r="G124" t="inlineStr"/>
+      <c r="H124" t="inlineStr"/>
+      <c r="I124" t="inlineStr"/>
+      <c r="J124" t="inlineStr"/>
+      <c r="K124" t="inlineStr">
         <is>
           <t>Catálogo: DIN 471 aço mola 60 mm (desenho: SAE 1070).</t>
         </is>
@@ -4553,7 +6432,11 @@
           <t>Comprado</t>
         </is>
       </c>
-      <c r="G125" t="inlineStr">
+      <c r="G125" t="inlineStr"/>
+      <c r="H125" t="inlineStr"/>
+      <c r="I125" t="inlineStr"/>
+      <c r="J125" t="inlineStr"/>
+      <c r="K125" t="inlineStr">
         <is>
           <t>CONFERIR: 3/8" fios de carbono e grafite flexível (cadastro em KG; desenho pede 3000 mm).</t>
         </is>
@@ -4588,7 +6471,11 @@
           <t>Comprado</t>
         </is>
       </c>
-      <c r="G126" t="inlineStr">
+      <c r="G126" t="inlineStr"/>
+      <c r="H126" t="inlineStr"/>
+      <c r="I126" t="inlineStr"/>
+      <c r="J126" t="inlineStr"/>
+      <c r="K126" t="inlineStr">
         <is>
           <t>Catálogo: DIN 976 Ø12 x 60 zincado preto.</t>
         </is>
@@ -4624,6 +6511,9 @@
         </is>
       </c>
       <c r="G127" t="inlineStr"/>
+      <c r="H127" t="inlineStr"/>
+      <c r="I127" t="inlineStr"/>
+      <c r="J127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -4655,6 +6545,9 @@
         </is>
       </c>
       <c r="G128" t="inlineStr"/>
+      <c r="H128" t="inlineStr"/>
+      <c r="I128" t="inlineStr"/>
+      <c r="J128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -4686,6 +6579,9 @@
         </is>
       </c>
       <c r="G129" t="inlineStr"/>
+      <c r="H129" t="inlineStr"/>
+      <c r="I129" t="inlineStr"/>
+      <c r="J129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -4717,6 +6613,9 @@
         </is>
       </c>
       <c r="G130" t="inlineStr"/>
+      <c r="H130" t="inlineStr"/>
+      <c r="I130" t="inlineStr"/>
+      <c r="J130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -4747,7 +6646,11 @@
           <t>Comprado</t>
         </is>
       </c>
-      <c r="G131" t="inlineStr">
+      <c r="G131" t="inlineStr"/>
+      <c r="H131" t="inlineStr"/>
+      <c r="I131" t="inlineStr"/>
+      <c r="J131" t="inlineStr"/>
+      <c r="K131" t="inlineStr">
         <is>
           <t>CONFERIR: cadastro CL 8.8 sem zincagem.</t>
         </is>
@@ -4783,6 +6686,9 @@
         </is>
       </c>
       <c r="G132" t="inlineStr"/>
+      <c r="H132" t="inlineStr"/>
+      <c r="I132" t="inlineStr"/>
+      <c r="J132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -4814,6 +6720,9 @@
         </is>
       </c>
       <c r="G133" t="inlineStr"/>
+      <c r="H133" t="inlineStr"/>
+      <c r="I133" t="inlineStr"/>
+      <c r="J133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -4845,6 +6754,9 @@
         </is>
       </c>
       <c r="G134" t="inlineStr"/>
+      <c r="H134" t="inlineStr"/>
+      <c r="I134" t="inlineStr"/>
+      <c r="J134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -4876,6 +6788,9 @@
         </is>
       </c>
       <c r="G135" t="inlineStr"/>
+      <c r="H135" t="inlineStr"/>
+      <c r="I135" t="inlineStr"/>
+      <c r="J135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -4906,7 +6821,11 @@
           <t>Comprado</t>
         </is>
       </c>
-      <c r="G136" t="inlineStr">
+      <c r="G136" t="inlineStr"/>
+      <c r="H136" t="inlineStr"/>
+      <c r="I136" t="inlineStr"/>
+      <c r="J136" t="inlineStr"/>
+      <c r="K136" t="inlineStr">
         <is>
           <t>CONFERIR: cadastro CL. 8 (não há Gr.8 M6).</t>
         </is>
@@ -4942,6 +6861,9 @@
         </is>
       </c>
       <c r="G137" t="inlineStr"/>
+      <c r="H137" t="inlineStr"/>
+      <c r="I137" t="inlineStr"/>
+      <c r="J137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -4972,7 +6894,11 @@
           <t>Comprado</t>
         </is>
       </c>
-      <c r="G138" t="inlineStr">
+      <c r="G138" t="inlineStr"/>
+      <c r="H138" t="inlineStr"/>
+      <c r="I138" t="inlineStr"/>
+      <c r="J138" t="inlineStr"/>
+      <c r="K138" t="inlineStr">
         <is>
           <t>CONFERIR: cadastro sem classe 8.8.</t>
         </is>
@@ -5008,6 +6934,9 @@
         </is>
       </c>
       <c r="G139" t="inlineStr"/>
+      <c r="H139" t="inlineStr"/>
+      <c r="I139" t="inlineStr"/>
+      <c r="J139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -5039,6 +6968,9 @@
         </is>
       </c>
       <c r="G140" t="inlineStr"/>
+      <c r="H140" t="inlineStr"/>
+      <c r="I140" t="inlineStr"/>
+      <c r="J140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -5070,6 +7002,9 @@
         </is>
       </c>
       <c r="G141" t="inlineStr"/>
+      <c r="H141" t="inlineStr"/>
+      <c r="I141" t="inlineStr"/>
+      <c r="J141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -5101,6 +7036,9 @@
         </is>
       </c>
       <c r="G142" t="inlineStr"/>
+      <c r="H142" t="inlineStr"/>
+      <c r="I142" t="inlineStr"/>
+      <c r="J142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -5132,6 +7070,9 @@
         </is>
       </c>
       <c r="G143" t="inlineStr"/>
+      <c r="H143" t="inlineStr"/>
+      <c r="I143" t="inlineStr"/>
+      <c r="J143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -5163,6 +7104,9 @@
         </is>
       </c>
       <c r="G144" t="inlineStr"/>
+      <c r="H144" t="inlineStr"/>
+      <c r="I144" t="inlineStr"/>
+      <c r="J144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -5194,6 +7138,9 @@
         </is>
       </c>
       <c r="G145" t="inlineStr"/>
+      <c r="H145" t="inlineStr"/>
+      <c r="I145" t="inlineStr"/>
+      <c r="J145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -5224,7 +7171,11 @@
           <t>Comprado</t>
         </is>
       </c>
-      <c r="G146" t="inlineStr">
+      <c r="G146" t="inlineStr"/>
+      <c r="H146" t="inlineStr"/>
+      <c r="I146" t="inlineStr"/>
+      <c r="J146" t="inlineStr"/>
+      <c r="K146" t="inlineStr">
         <is>
           <t>CONFERIR: há também 01.13.3.18 (classe #150).</t>
         </is>
@@ -5259,7 +7210,11 @@
           <t>Comprado</t>
         </is>
       </c>
-      <c r="G147" t="inlineStr">
+      <c r="G147" t="inlineStr"/>
+      <c r="H147" t="inlineStr"/>
+      <c r="I147" t="inlineStr"/>
+      <c r="J147" t="inlineStr"/>
+      <c r="K147" t="inlineStr">
         <is>
           <t>CONFERIR: cadastro é 1" NPT ASTM A197; desenho diz rosca BSP.</t>
         </is>
@@ -5295,6 +7250,9 @@
         </is>
       </c>
       <c r="G148" t="inlineStr"/>
+      <c r="H148" t="inlineStr"/>
+      <c r="I148" t="inlineStr"/>
+      <c r="J148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -5326,6 +7284,9 @@
         </is>
       </c>
       <c r="G149" t="inlineStr"/>
+      <c r="H149" t="inlineStr"/>
+      <c r="I149" t="inlineStr"/>
+      <c r="J149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -5357,6 +7318,9 @@
         </is>
       </c>
       <c r="G150" t="inlineStr"/>
+      <c r="H150" t="inlineStr"/>
+      <c r="I150" t="inlineStr"/>
+      <c r="J150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -5388,6 +7352,9 @@
         </is>
       </c>
       <c r="G151" t="inlineStr"/>
+      <c r="H151" t="inlineStr"/>
+      <c r="I151" t="inlineStr"/>
+      <c r="J151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -5419,6 +7386,9 @@
         </is>
       </c>
       <c r="G152" t="inlineStr"/>
+      <c r="H152" t="inlineStr"/>
+      <c r="I152" t="inlineStr"/>
+      <c r="J152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -5449,7 +7419,11 @@
           <t>Comprado</t>
         </is>
       </c>
-      <c r="G153" t="inlineStr">
+      <c r="G153" t="inlineStr"/>
+      <c r="H153" t="inlineStr"/>
+      <c r="I153" t="inlineStr"/>
+      <c r="J153" t="inlineStr"/>
+      <c r="K153" t="inlineStr">
         <is>
           <t>CONFERIR: há também 01.13.1.13.10.10. Qtd em mm (6000).</t>
         </is>
@@ -5485,6 +7459,9 @@
         </is>
       </c>
       <c r="G154" t="inlineStr"/>
+      <c r="H154" t="inlineStr"/>
+      <c r="I154" t="inlineStr"/>
+      <c r="J154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -5516,6 +7493,9 @@
         </is>
       </c>
       <c r="G155" t="inlineStr"/>
+      <c r="H155" t="inlineStr"/>
+      <c r="I155" t="inlineStr"/>
+      <c r="J155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -5546,7 +7526,11 @@
           <t>Comprado</t>
         </is>
       </c>
-      <c r="G156" t="inlineStr">
+      <c r="G156" t="inlineStr"/>
+      <c r="H156" t="inlineStr"/>
+      <c r="I156" t="inlineStr"/>
+      <c r="J156" t="inlineStr"/>
+      <c r="K156" t="inlineStr">
         <is>
           <t>CONFERIR: 1/4" carbono com grafite flexível (cadastro em KG; desenho pede 900 mm).</t>
         </is>
@@ -5582,6 +7566,9 @@
         </is>
       </c>
       <c r="G157" t="inlineStr"/>
+      <c r="H157" t="inlineStr"/>
+      <c r="I157" t="inlineStr"/>
+      <c r="J157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
@@ -5589,20 +7576,24 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="B158" s="4" t="inlineStr"/>
+      <c r="B158" s="4" t="n"/>
       <c r="C158" s="4" t="inlineStr">
         <is>
           <t>[DEFINIR] Item do balão 52 (aparece no desenho 022-007300, sem linha na lista)</t>
         </is>
       </c>
-      <c r="D158" s="4" t="inlineStr"/>
-      <c r="E158" s="4" t="inlineStr"/>
+      <c r="D158" s="4" t="n"/>
+      <c r="E158" s="4" t="n"/>
       <c r="F158" s="4" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="G158" s="4" t="inlineStr">
+      <c r="G158" s="4" t="inlineStr"/>
+      <c r="H158" s="4" t="inlineStr"/>
+      <c r="I158" s="4" t="inlineStr"/>
+      <c r="J158" s="4" t="inlineStr"/>
+      <c r="K158" s="4" t="inlineStr">
         <is>
           <t>Sem descrição na lista do desenho</t>
         </is>
@@ -5614,20 +7605,24 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="B159" s="4" t="inlineStr"/>
+      <c r="B159" s="4" t="n"/>
       <c r="C159" s="4" t="inlineStr">
         <is>
           <t>[DEFINIR] Item do balão 62 (aparece no desenho 022-007300, sem linha na lista)</t>
         </is>
       </c>
-      <c r="D159" s="4" t="inlineStr"/>
-      <c r="E159" s="4" t="inlineStr"/>
+      <c r="D159" s="4" t="n"/>
+      <c r="E159" s="4" t="n"/>
       <c r="F159" s="4" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="G159" s="4" t="inlineStr">
+      <c r="G159" s="4" t="inlineStr"/>
+      <c r="H159" s="4" t="inlineStr"/>
+      <c r="I159" s="4" t="inlineStr"/>
+      <c r="J159" s="4" t="inlineStr"/>
+      <c r="K159" s="4" t="inlineStr">
         <is>
           <t>Sem descrição na lista do desenho</t>
         </is>
@@ -5639,27 +7634,31 @@
           <t>04.01.3.000598</t>
         </is>
       </c>
-      <c r="B160" s="4" t="inlineStr"/>
+      <c r="B160" s="4" t="n"/>
       <c r="C160" s="4" t="inlineStr">
         <is>
           <t>[DEFINIR] Item do balão 65 (aparece no desenho 022-007300, sem linha na lista)</t>
         </is>
       </c>
-      <c r="D160" s="4" t="inlineStr"/>
-      <c r="E160" s="4" t="inlineStr"/>
+      <c r="D160" s="4" t="n"/>
+      <c r="E160" s="4" t="n"/>
       <c r="F160" s="4" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="G160" s="4" t="inlineStr">
+      <c r="G160" s="4" t="inlineStr"/>
+      <c r="H160" s="4" t="inlineStr"/>
+      <c r="I160" s="4" t="inlineStr"/>
+      <c r="J160" s="4" t="inlineStr"/>
+      <c r="K160" s="4" t="inlineStr">
         <is>
           <t>Sem descrição na lista do desenho</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G160"/>
+  <autoFilter ref="A1:K160"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10560,7 +12559,6 @@
         </is>
       </c>
     </row>
-    <row r="123"/>
     <row r="124">
       <c r="C124" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix plate thickness parsing
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019oxoH766RXuqLqXQEjeJHj
</commit_message>
<xml_diff>
--- a/Estrutura_04.01.3.000598.xlsx
+++ b/Estrutura_04.01.3.000598.xlsx
@@ -1060,11 +1060,11 @@
         </is>
       </c>
       <c r="H15" s="5" t="n">
-        <v>1793.88</v>
+        <v>15.88</v>
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>chapa 70 5/8"</t>
+          <t>chapa 5/8"</t>
         </is>
       </c>
       <c r="J15" s="5" t="n">
@@ -1144,11 +1144,11 @@
         </is>
       </c>
       <c r="H17" s="5" t="n">
-        <v>1797.05</v>
+        <v>19.05</v>
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>chapa 70 3/4"</t>
+          <t>chapa 3/4"</t>
         </is>
       </c>
       <c r="J17" s="5" t="n">
@@ -1765,11 +1765,11 @@
         </is>
       </c>
       <c r="H32" s="5" t="n">
-        <v>1790.7</v>
+        <v>12.7</v>
       </c>
       <c r="I32" s="5" t="inlineStr">
         <is>
-          <t>chapa 70 1/2"</t>
+          <t>chapa 1/2"</t>
         </is>
       </c>
       <c r="J32" s="5" t="n">
@@ -3314,11 +3314,11 @@
         </is>
       </c>
       <c r="H70" s="5" t="n">
-        <v>1793.88</v>
+        <v>15.88</v>
       </c>
       <c r="I70" s="5" t="inlineStr">
         <is>
-          <t>chapa 70 5/8"</t>
+          <t>chapa 5/8"</t>
         </is>
       </c>
       <c r="J70" s="5" t="n">
@@ -3457,11 +3457,11 @@
         </is>
       </c>
       <c r="H74" s="5" t="n">
-        <v>1790.7</v>
+        <v>12.7</v>
       </c>
       <c r="I74" s="5" t="inlineStr">
         <is>
-          <t>chapa 70 1/2"</t>
+          <t>chapa 1/2"</t>
         </is>
       </c>
       <c r="J74" s="5" t="n">
@@ -3691,11 +3691,11 @@
         </is>
       </c>
       <c r="H80" s="5" t="n">
-        <v>1790.7</v>
+        <v>12.7</v>
       </c>
       <c r="I80" s="5" t="inlineStr">
         <is>
-          <t>chapa 70 1/2"</t>
+          <t>chapa 1/2"</t>
         </is>
       </c>
       <c r="J80" s="5" t="n">
@@ -3775,11 +3775,11 @@
         </is>
       </c>
       <c r="H82" s="5" t="n">
-        <v>1793.88</v>
+        <v>15.88</v>
       </c>
       <c r="I82" s="5" t="inlineStr">
         <is>
-          <t>chapa 70 5/8"</t>
+          <t>chapa 5/8"</t>
         </is>
       </c>
       <c r="J82" s="5" t="n">
@@ -4200,11 +4200,11 @@
         </is>
       </c>
       <c r="H92" s="5" t="n">
-        <v>1793.88</v>
+        <v>15.88</v>
       </c>
       <c r="I92" s="5" t="inlineStr">
         <is>
-          <t>chapa 70 5/8"</t>
+          <t>chapa 5/8"</t>
         </is>
       </c>
       <c r="J92" s="5" t="n">
@@ -4368,11 +4368,11 @@
         </is>
       </c>
       <c r="H96" s="5" t="n">
-        <v>1790.7</v>
+        <v>12.7</v>
       </c>
       <c r="I96" s="5" t="inlineStr">
         <is>
-          <t>chapa 70 1/2"</t>
+          <t>chapa 1/2"</t>
         </is>
       </c>
       <c r="J96" s="5" t="n">
@@ -4536,11 +4536,11 @@
         </is>
       </c>
       <c r="H100" s="5" t="n">
-        <v>1790.7</v>
+        <v>12.7</v>
       </c>
       <c r="I100" s="5" t="inlineStr">
         <is>
-          <t>chapa 70 1/2"</t>
+          <t>chapa 1/2"</t>
         </is>
       </c>
       <c r="J100" s="5" t="n">
@@ -5434,11 +5434,11 @@
         </is>
       </c>
       <c r="H122" s="5" t="n">
-        <v>1793.88</v>
+        <v>15.88</v>
       </c>
       <c r="I122" s="5" t="inlineStr">
         <is>
-          <t>chapa 70 5/8"</t>
+          <t>chapa 5/8"</t>
         </is>
       </c>
       <c r="J122" s="5" t="n">

</xml_diff>